<commit_message>
Fix Golpayegan district detection and multi-location report scanning: support root/subfolder/program directory scanning, robust cell/sheet search, English transliterations, and Persian comma parsing
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/final_scores.xlsx
+++ b/final_scores.xlsx
@@ -71,7 +71,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -100,18 +100,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FEE2E2"/>
         <bgColor rgb="00FEE2E2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FEF3C7"/>
-        <bgColor rgb="00FEF3C7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D1FAE5"/>
-        <bgColor rgb="00D1FAE5"/>
       </patternFill>
     </fill>
     <fill>
@@ -147,7 +135,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -179,13 +167,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -568,7 +550,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>نمره نسرا (۷۰-۱۰۰)</t>
+          <t>نمره واقعی (۰-۱۰۰)</t>
         </is>
       </c>
     </row>
@@ -579,7 +561,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -589,7 +571,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -599,7 +581,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -609,7 +591,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -619,7 +601,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -629,7 +611,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -639,7 +621,7 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>85.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -649,7 +631,7 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -659,7 +641,7 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -669,7 +651,7 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -679,7 +661,7 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -689,7 +671,7 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -699,7 +681,7 @@
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -709,7 +691,7 @@
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -719,7 +701,7 @@
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>97.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -729,7 +711,7 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -739,7 +721,7 @@
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -749,7 +731,7 @@
         </is>
       </c>
       <c r="B19" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -759,7 +741,7 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -769,7 +751,7 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -779,7 +761,7 @@
         </is>
       </c>
       <c r="B22" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -789,7 +771,7 @@
         </is>
       </c>
       <c r="B23" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -799,7 +781,7 @@
         </is>
       </c>
       <c r="B24" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -809,7 +791,7 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -819,7 +801,7 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -829,7 +811,7 @@
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -839,7 +821,7 @@
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -849,7 +831,7 @@
         </is>
       </c>
       <c r="B29" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -859,7 +841,7 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -869,7 +851,7 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -879,7 +861,7 @@
         </is>
       </c>
       <c r="B32" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -889,7 +871,7 @@
         </is>
       </c>
       <c r="B33" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1191,27 +1173,29 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>52.8</v>
+        <v>0</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>85.8</v>
-      </c>
-      <c r="E10" s="11" t="inlineStr">
-        <is>
-          <t>متوسط</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="n">
-        <v>2</v>
+        <v>70</v>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>ضعیف</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>52.8%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="H10" s="10" t="inlineStr">
         <is>
-          <t>کسری: 1 از 2 ماه (عدم فعالیت در: مرداد 1405)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
         </is>
       </c>
     </row>
@@ -1477,27 +1461,29 @@
         </is>
       </c>
       <c r="C18" s="7" t="n">
-        <v>90.8</v>
+        <v>0</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>97.2</v>
-      </c>
-      <c r="E18" s="12" t="inlineStr">
-        <is>
-          <t>عالی</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="n">
-        <v>1</v>
+        <v>70</v>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>ضعیف</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>90.8%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="H18" s="10" t="inlineStr">
         <is>
-          <t>کامل (2 از 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
         </is>
       </c>
     </row>
@@ -2142,7 +2128,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>جدول ارزیابی عملکرد ۲ ماهه نواحی نسرا (مقیاس استاندارد نسرا (۷۰ تا ۱۰۰))</t>
+          <t>جدول ارزیابی عملکرد ۲ ماهه نواحی نسرا (مقیاس واقعی (۰ تا ۱۰۰))</t>
         </is>
       </c>
     </row>
@@ -2159,7 +2145,7 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>نمره نسرا (۷۰-۱۰۰)</t>
+          <t>نمره واقعی (۰-۱۰۰)</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
@@ -2193,7 +2179,7 @@
         </is>
       </c>
       <c r="C4" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
@@ -2226,7 +2212,7 @@
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
@@ -2259,7 +2245,7 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
@@ -2292,7 +2278,7 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
@@ -2325,7 +2311,7 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
@@ -2358,7 +2344,7 @@
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
@@ -2391,24 +2377,26 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>85.8</v>
-      </c>
-      <c r="D10" s="11" t="inlineStr">
-        <is>
-          <t>متوسط</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="n">
-        <v>2</v>
+        <v>0</v>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>ضعیف</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>1 از 2 ماه</t>
+          <t>0 از 2 ماه</t>
         </is>
       </c>
       <c r="G10" s="10" t="inlineStr">
         <is>
-          <t>کسری: 1 از 2 ماه (عدم فعالیت در: مرداد 1405)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
         </is>
       </c>
     </row>
@@ -2422,7 +2410,7 @@
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
@@ -2455,7 +2443,7 @@
         </is>
       </c>
       <c r="C12" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
@@ -2488,7 +2476,7 @@
         </is>
       </c>
       <c r="C13" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
@@ -2521,7 +2509,7 @@
         </is>
       </c>
       <c r="C14" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
@@ -2554,7 +2542,7 @@
         </is>
       </c>
       <c r="C15" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
@@ -2587,7 +2575,7 @@
         </is>
       </c>
       <c r="C16" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
@@ -2620,7 +2608,7 @@
         </is>
       </c>
       <c r="C17" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
@@ -2653,24 +2641,26 @@
         </is>
       </c>
       <c r="C18" s="7" t="n">
-        <v>97.2</v>
-      </c>
-      <c r="D18" s="12" t="inlineStr">
-        <is>
-          <t>عالی</t>
-        </is>
-      </c>
-      <c r="E18" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>ضعیف</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>2 از 2 ماه</t>
+          <t>0 از 2 ماه</t>
         </is>
       </c>
       <c r="G18" s="10" t="inlineStr">
         <is>
-          <t>کامل (2 از 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
         </is>
       </c>
     </row>
@@ -2684,7 +2674,7 @@
         </is>
       </c>
       <c r="C19" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
@@ -2717,7 +2707,7 @@
         </is>
       </c>
       <c r="C20" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
@@ -2750,7 +2740,7 @@
         </is>
       </c>
       <c r="C21" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
@@ -2783,7 +2773,7 @@
         </is>
       </c>
       <c r="C22" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
@@ -2816,7 +2806,7 @@
         </is>
       </c>
       <c r="C23" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
@@ -2849,7 +2839,7 @@
         </is>
       </c>
       <c r="C24" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
@@ -2882,7 +2872,7 @@
         </is>
       </c>
       <c r="C25" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
@@ -2915,7 +2905,7 @@
         </is>
       </c>
       <c r="C26" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
@@ -2948,7 +2938,7 @@
         </is>
       </c>
       <c r="C27" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
@@ -2981,7 +2971,7 @@
         </is>
       </c>
       <c r="C28" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
@@ -3014,7 +3004,7 @@
         </is>
       </c>
       <c r="C29" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
@@ -3047,7 +3037,7 @@
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
@@ -3080,7 +3070,7 @@
         </is>
       </c>
       <c r="C31" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
@@ -3113,7 +3103,7 @@
         </is>
       </c>
       <c r="C32" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
@@ -3146,7 +3136,7 @@
         </is>
       </c>
       <c r="C33" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
@@ -3179,7 +3169,7 @@
         </is>
       </c>
       <c r="C34" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
@@ -3212,7 +3202,7 @@
         </is>
       </c>
       <c r="C35" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
@@ -3264,106 +3254,110 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>رتبه‌بندی استانی عملکرد ۲ ماهه ۳۲ شهرستان (مقیاس استاندارد نسرا (۷۰ تا ۱۰۰))</t>
+          <t>رتبه‌بندی استانی عملکرد ۲ ماهه ۳۲ شهرستان (مقیاس واقعی (۰ تا ۱۰۰))</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>رتبه</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>نام ناحیه (شهرستان)</t>
         </is>
       </c>
-      <c r="C3" s="13" t="inlineStr">
-        <is>
-          <t>نمره نسرا (۷۰-۱۰۰)</t>
-        </is>
-      </c>
-      <c r="D3" s="13" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
+        <is>
+          <t>نمره واقعی (۰-۱۰۰)</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
         <is>
           <t>نمره مقیاس دیگر</t>
         </is>
       </c>
-      <c r="E3" s="13" t="inlineStr">
+      <c r="E3" s="11" t="inlineStr">
         <is>
           <t>سطح کیفی</t>
         </is>
       </c>
-      <c r="F3" s="13" t="inlineStr">
+      <c r="F3" s="11" t="inlineStr">
         <is>
           <t>درصد تحقق وزنی</t>
         </is>
       </c>
-      <c r="G3" s="13" t="inlineStr">
+      <c r="G3" s="11" t="inlineStr">
         <is>
           <t>تعداد ماه‌های ارسالی</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="n">
-        <v>1</v>
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>درچه</t>
+          <t>آران و بیدگل</t>
         </is>
       </c>
       <c r="C4" s="7" t="n">
-        <v>97.2</v>
+        <v>0</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>90.8</v>
-      </c>
-      <c r="E4" s="12" t="inlineStr">
-        <is>
-          <t>عالی</t>
+        <v>70</v>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>ضعیف</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>90.8%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>2 از 2 ماه</t>
+          <t>0 از 2 ماه</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="n">
-        <v>2</v>
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>برخوار</t>
+          <t>امام حسین(ع)</t>
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>85.8</v>
+        <v>0</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>52.8</v>
-      </c>
-      <c r="E5" s="11" t="inlineStr">
-        <is>
-          <t>متوسط</t>
+        <v>70</v>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>ضعیف</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>52.8%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>1 از 2 ماه</t>
+          <t>0 از 2 ماه</t>
         </is>
       </c>
     </row>
@@ -3375,14 +3369,14 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>آران و بیدگل</t>
+          <t>امام رضا(ع)</t>
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
@@ -3408,14 +3402,14 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>امام حسین(ع)</t>
+          <t>امام صادق(ع)</t>
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
@@ -3441,14 +3435,14 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>امام رضا(ع)</t>
+          <t>امام علی(ع)</t>
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
@@ -3474,14 +3468,14 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>امام صادق(ع)</t>
+          <t>اردستان</t>
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
@@ -3507,14 +3501,14 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>امام علی(ع)</t>
+          <t>برخوار</t>
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
@@ -3540,14 +3534,14 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>اردستان</t>
+          <t>بویین و میاندشت</t>
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
@@ -3573,14 +3567,14 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>بویین و میاندشت</t>
+          <t>تیران و کرون</t>
         </is>
       </c>
       <c r="C12" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
@@ -3606,14 +3600,14 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>تیران و کرون</t>
+          <t>جرقویه</t>
         </is>
       </c>
       <c r="C13" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
@@ -3639,14 +3633,14 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>جرقویه</t>
+          <t>چادگان</t>
         </is>
       </c>
       <c r="C14" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
@@ -3672,14 +3666,14 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>چادگان</t>
+          <t>خمینی شهر</t>
         </is>
       </c>
       <c r="C15" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D15" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
@@ -3705,14 +3699,14 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>خمینی شهر</t>
+          <t>خوانسار</t>
         </is>
       </c>
       <c r="C16" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
@@ -3738,14 +3732,14 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>خوانسار</t>
+          <t>خور و بیابانک</t>
         </is>
       </c>
       <c r="C17" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D17" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
@@ -3771,14 +3765,14 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>خور و بیابانک</t>
+          <t>درچه</t>
         </is>
       </c>
       <c r="C18" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
@@ -3808,10 +3802,10 @@
         </is>
       </c>
       <c r="C19" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D19" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
@@ -3841,10 +3835,10 @@
         </is>
       </c>
       <c r="C20" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D20" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
@@ -3874,10 +3868,10 @@
         </is>
       </c>
       <c r="C21" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D21" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
@@ -3907,10 +3901,10 @@
         </is>
       </c>
       <c r="C22" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D22" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
@@ -3940,10 +3934,10 @@
         </is>
       </c>
       <c r="C23" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
@@ -3973,10 +3967,10 @@
         </is>
       </c>
       <c r="C24" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
@@ -4006,10 +4000,10 @@
         </is>
       </c>
       <c r="C25" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
@@ -4039,10 +4033,10 @@
         </is>
       </c>
       <c r="C26" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D26" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
@@ -4072,10 +4066,10 @@
         </is>
       </c>
       <c r="C27" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D27" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
@@ -4105,10 +4099,10 @@
         </is>
       </c>
       <c r="C28" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D28" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
@@ -4138,10 +4132,10 @@
         </is>
       </c>
       <c r="C29" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D29" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
@@ -4171,10 +4165,10 @@
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D30" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
@@ -4204,10 +4198,10 @@
         </is>
       </c>
       <c r="C31" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D31" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
@@ -4237,10 +4231,10 @@
         </is>
       </c>
       <c r="C32" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D32" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
@@ -4270,10 +4264,10 @@
         </is>
       </c>
       <c r="C33" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D33" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
@@ -4303,10 +4297,10 @@
         </is>
       </c>
       <c r="C34" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D34" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
@@ -4336,10 +4330,10 @@
         </is>
       </c>
       <c r="C35" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D35" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
@@ -4405,107 +4399,107 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>ردیف</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>نام ناحیه</t>
         </is>
       </c>
-      <c r="C3" s="13" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>نمره واقعی (۰-۱۰۰)</t>
         </is>
       </c>
-      <c r="D3" s="13" t="inlineStr">
+      <c r="D3" s="11" t="inlineStr">
         <is>
           <t>نمره نسرا (۷۰-۱۰۰)</t>
         </is>
       </c>
-      <c r="E3" s="13" t="inlineStr">
+      <c r="E3" s="11" t="inlineStr">
         <is>
           <t>سطح</t>
         </is>
       </c>
-      <c r="F3" s="13" t="inlineStr">
+      <c r="F3" s="11" t="inlineStr">
         <is>
           <t>رتبه</t>
         </is>
       </c>
-      <c r="G3" s="13" t="inlineStr">
+      <c r="G3" s="11" t="inlineStr">
         <is>
           <t>ماه‌ها</t>
         </is>
       </c>
-      <c r="H3" s="13" t="inlineStr">
+      <c r="H3" s="11" t="inlineStr">
         <is>
           <t>حوزه</t>
         </is>
       </c>
-      <c r="I3" s="13" t="inlineStr">
+      <c r="I3" s="11" t="inlineStr">
         <is>
           <t>انتظار حضوری</t>
         </is>
       </c>
-      <c r="J3" s="13" t="inlineStr">
+      <c r="J3" s="11" t="inlineStr">
         <is>
           <t>عملکرد حضوری</t>
         </is>
       </c>
-      <c r="K3" s="13" t="inlineStr">
+      <c r="K3" s="11" t="inlineStr">
         <is>
           <t>تحقق حضوری</t>
         </is>
       </c>
-      <c r="L3" s="13" t="inlineStr">
+      <c r="L3" s="11" t="inlineStr">
         <is>
           <t>انتظار مجازی</t>
         </is>
       </c>
-      <c r="M3" s="13" t="inlineStr">
+      <c r="M3" s="11" t="inlineStr">
         <is>
           <t>عملکرد مجازی</t>
         </is>
       </c>
-      <c r="N3" s="13" t="inlineStr">
+      <c r="N3" s="11" t="inlineStr">
         <is>
           <t>تحقق مجازی</t>
         </is>
       </c>
-      <c r="O3" s="13" t="inlineStr">
+      <c r="O3" s="11" t="inlineStr">
         <is>
           <t>سهم آموزش (۴۰٪)</t>
         </is>
       </c>
-      <c r="P3" s="13" t="inlineStr">
+      <c r="P3" s="11" t="inlineStr">
         <is>
           <t>انتظار خلاقانه</t>
         </is>
       </c>
-      <c r="Q3" s="13" t="inlineStr">
+      <c r="Q3" s="11" t="inlineStr">
         <is>
           <t>عملکرد خلاقانه</t>
         </is>
       </c>
-      <c r="R3" s="13" t="inlineStr">
+      <c r="R3" s="11" t="inlineStr">
         <is>
           <t>سهم خلاقانه (۵۰٪)</t>
         </is>
       </c>
-      <c r="S3" s="13" t="inlineStr">
+      <c r="S3" s="11" t="inlineStr">
         <is>
           <t>انتظار تولید</t>
         </is>
       </c>
-      <c r="T3" s="13" t="inlineStr">
+      <c r="T3" s="11" t="inlineStr">
         <is>
           <t>عملکرد تولید</t>
         </is>
       </c>
-      <c r="U3" s="13" t="inlineStr">
+      <c r="U3" s="11" t="inlineStr">
         <is>
           <t>سهم تولید (۱۰٪)</t>
         </is>
@@ -5019,22 +5013,24 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>52.8</v>
+        <v>0</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>85.8</v>
+        <v>70</v>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>متوسط</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="n">
-        <v>2</v>
+          <t>ضعیف</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>1 از 2</t>
+          <t>0 از 2</t>
         </is>
       </c>
       <c r="H10" s="6" t="n">
@@ -5044,18 +5040,18 @@
         <v>310</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
-          <t>14.8%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="L10" s="6" t="n">
         <v>2170</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N10" s="6" t="inlineStr">
         <is>
@@ -5064,29 +5060,29 @@
       </c>
       <c r="O10" s="6" t="inlineStr">
         <is>
-          <t>1.50%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P10" s="6" t="n">
         <v>620</v>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>4396</v>
+        <v>0</v>
       </c>
       <c r="R10" s="6" t="inlineStr">
         <is>
-          <t>50.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="S10" s="6" t="n">
         <v>30</v>
       </c>
       <c r="T10" s="6" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="U10" s="6" t="inlineStr">
         <is>
-          <t>1.33%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -5681,22 +5677,24 @@
         </is>
       </c>
       <c r="C18" s="7" t="n">
-        <v>90.8</v>
+        <v>0</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>97.2</v>
+        <v>70</v>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>عالی</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="n">
-        <v>1</v>
+          <t>ضعیف</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>2 از 2</t>
+          <t>0 از 2</t>
         </is>
       </c>
       <c r="H18" s="6" t="n">
@@ -5706,49 +5704,49 @@
         <v>248</v>
       </c>
       <c r="J18" s="6" t="n">
-        <v>4552</v>
+        <v>0</v>
       </c>
       <c r="K18" s="6" t="inlineStr">
         <is>
-          <t>1835.5%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="L18" s="6" t="n">
         <v>1736</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N18" s="6" t="inlineStr">
         <is>
-          <t>0.1%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="O18" s="6" t="inlineStr">
         <is>
-          <t>40.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P18" s="6" t="n">
         <v>496</v>
       </c>
       <c r="Q18" s="6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R18" s="6" t="inlineStr">
         <is>
-          <t>50.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="S18" s="6" t="n">
         <v>24</v>
       </c>
       <c r="T18" s="6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U18" s="6" t="inlineStr">
         <is>
-          <t>0.83%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>

</xml_diff>